<commit_message>
Finalize Dropline QC and organize run evidence
Harden the Dropline v6.0.1 golden solution and browser verifiers, refresh the Brickfall v1.0.1 baseline and deliverable, and preserve platform run evidence under shorter outer paths.
</commit_message>
<xml_diff>
--- a/projects/dropline-four-lite/environment/assets/artifacts/dropline_seed.xlsx
+++ b/projects/dropline-four-lite/environment/assets/artifacts/dropline_seed.xlsx
@@ -1,50 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
-  <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
-  </bookViews>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Accounts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Initial Game State" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Accounts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Initial Game State" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Completed Matches" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Accounts'!$A$1:$C$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Initial Game State'!$A$1:$H$3</definedName>
-  </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <definedNames/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001D62A0"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -59,19 +43,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -218,6 +196,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -252,6 +231,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -286,20 +266,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -421,7 +397,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -434,65 +449,59 @@
   </sheetPr>
   <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Password</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>avery@dropline.test</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>password123</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Avery Morgan</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>jordan@dropline.test</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>password123</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Jordan Lee</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -503,135 +512,578 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Account email</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Board</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Current player</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Winning cells</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Red wins</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Yellow wins</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Draws</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Applied history</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Redo history</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Revision</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Round id</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>avery@dropline.test</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>42 empty cells</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>["","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","Red","Yellow","",""]</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":4,"row":6,"index":38},{"color":"Yellow","column":5,"row":6,"index":39}]</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":4,"row":5,"index":31}]</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>7</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>seed-avery-midgame</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>["","","","","","","","","","","","","","","","","","","","","","","","","","","","","","Red","","","","","","","Red","Yellow","","","",""]</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Yellow</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>0</v>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":2,"row":6,"index":36},{"color":"Yellow","column":3,"row":6,"index":37},{"color":"Red","column":2,"row":5,"index":29}]</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>seed-jordan-active</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Account email</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Match id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Final board</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Moves</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Completed at</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>seed-jordan-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Red wins</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>["","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","Yellow","Red","Red","Red","Red","","Yellow","Yellow"]</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":1,"row":6,"index":35},{"color":"Yellow","column":7,"row":6,"index":41},{"color":"Red","column":2,"row":6,"index":36},{"color":"Yellow","column":7,"row":5,"index":34},{"color":"Red","column":3,"row":6,"index":37},{"color":"Yellow","column":6,"row":6,"index":40},{"color":"Red","column":4,"row":6,"index":38}]</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-01-01T10:00:00.000Z</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>jordan@dropline.test</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>42 empty cells</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>0</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>seed-jordan-02</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Yellow wins</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>["","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","Red","Red","Yellow","Yellow","Yellow","Yellow","","Red","Red"]</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":7,"row":6,"index":41},{"color":"Yellow","column":1,"row":6,"index":35},{"color":"Red","column":7,"row":5,"index":34},{"color":"Yellow","column":2,"row":6,"index":36},{"color":"Red","column":6,"row":6,"index":40},{"color":"Yellow","column":3,"row":6,"index":37},{"color":"Red","column":6,"row":5,"index":33},{"color":"Yellow","column":4,"row":6,"index":38}]</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-01-02T10:00:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>seed-jordan-03</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>["Yellow","Red","Yellow","Yellow","Yellow","Red","Yellow","Red","Yellow","Red","Red","Red","Yellow","Red","Yellow","Red","Yellow","Yellow","Yellow","Red","Yellow","Red","Yellow","Red","Red","Red","Yellow","Red","Yellow","Red","Yellow","Yellow","Red","Yellow","Yellow","Red","Yellow","Red","Red","Red","Yellow","Red"]</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":4,"row":6,"index":38},{"color":"Yellow","column":4,"row":5,"index":31},{"color":"Red","column":4,"row":4,"index":24},{"color":"Yellow","column":4,"row":3,"index":17},{"color":"Red","column":4,"row":2,"index":10},{"color":"Yellow","column":4,"row":1,"index":3},{"color":"Red","column":3,"row":6,"index":37},{"color":"Yellow","column":3,"row":5,"index":30},{"color":"Red","column":3,"row":4,"index":23},{"color":"Yellow","column":3,"row":3,"index":16},{"color":"Red","column":3,"row":2,"index":9},{"color":"Yellow","column":3,"row":1,"index":2},{"color":"Red","column":5,"row":6,"index":39},{"color":"Yellow","column":2,"row":6,"index":36},{"color":"Red","column":5,"row":5,"index":32},{"color":"Yellow","column":6,"row":6,"index":40},{"color":"Red","column":5,"row":4,"index":25},{"color":"Yellow","column":5,"row":3,"index":18},{"color":"Red","column":5,"row":2,"index":11},{"color":"Yellow","column":5,"row":1,"index":4},{"color":"Red","column":2,"row":5,"index":29},{"color":"Yellow","column":2,"row":4,"index":22},{"color":"Red","column":2,"row":3,"index":15},{"color":"Yellow","column":2,"row":2,"index":8},{"color":"Red","column":2,"row":1,"index":1},{"color":"Yellow","column":6,"row":5,"index":33},{"color":"Red","column":1,"row":6,"index":35},{"color":"Yellow","column":6,"row":4,"index":26},{"color":"Red","column":6,"row":3,"index":19},{"color":"Yellow","column":6,"row":2,"index":12},{"color":"Red","column":6,"row":1,"index":5},{"color":"Yellow","column":1,"row":5,"index":28},{"color":"Red","column":1,"row":4,"index":21},{"color":"Yellow","column":1,"row":3,"index":14},{"color":"Red","column":1,"row":2,"index":7},{"color":"Yellow","column":1,"row":1,"index":0},{"color":"Red","column":7,"row":6,"index":41},{"color":"Yellow","column":7,"row":5,"index":34},{"color":"Red","column":7,"row":4,"index":27},{"color":"Yellow","column":7,"row":3,"index":20},{"color":"Red","column":7,"row":2,"index":13},{"color":"Yellow","column":7,"row":1,"index":6}]</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-01-03T10:00:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>seed-jordan-04</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Red wins</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>["","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","Yellow","Red","Red","Red","Red","","Yellow","Yellow"]</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":1,"row":6,"index":35},{"color":"Yellow","column":7,"row":6,"index":41},{"color":"Red","column":2,"row":6,"index":36},{"color":"Yellow","column":7,"row":5,"index":34},{"color":"Red","column":3,"row":6,"index":37},{"color":"Yellow","column":6,"row":6,"index":40},{"color":"Red","column":4,"row":6,"index":38}]</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-01-04T10:00:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>seed-jordan-05</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Yellow wins</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>["","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","Red","Red","Yellow","Yellow","Yellow","Yellow","","Red","Red"]</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":7,"row":6,"index":41},{"color":"Yellow","column":1,"row":6,"index":35},{"color":"Red","column":7,"row":5,"index":34},{"color":"Yellow","column":2,"row":6,"index":36},{"color":"Red","column":6,"row":6,"index":40},{"color":"Yellow","column":3,"row":6,"index":37},{"color":"Red","column":6,"row":5,"index":33},{"color":"Yellow","column":4,"row":6,"index":38}]</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-01-05T10:00:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>seed-jordan-06</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>["Yellow","Red","Yellow","Yellow","Yellow","Red","Yellow","Red","Yellow","Red","Red","Red","Yellow","Red","Yellow","Red","Yellow","Yellow","Yellow","Red","Yellow","Red","Yellow","Red","Red","Red","Yellow","Red","Yellow","Red","Yellow","Yellow","Red","Yellow","Yellow","Red","Yellow","Red","Red","Red","Yellow","Red"]</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":4,"row":6,"index":38},{"color":"Yellow","column":4,"row":5,"index":31},{"color":"Red","column":4,"row":4,"index":24},{"color":"Yellow","column":4,"row":3,"index":17},{"color":"Red","column":4,"row":2,"index":10},{"color":"Yellow","column":4,"row":1,"index":3},{"color":"Red","column":3,"row":6,"index":37},{"color":"Yellow","column":3,"row":5,"index":30},{"color":"Red","column":3,"row":4,"index":23},{"color":"Yellow","column":3,"row":3,"index":16},{"color":"Red","column":3,"row":2,"index":9},{"color":"Yellow","column":3,"row":1,"index":2},{"color":"Red","column":5,"row":6,"index":39},{"color":"Yellow","column":2,"row":6,"index":36},{"color":"Red","column":5,"row":5,"index":32},{"color":"Yellow","column":6,"row":6,"index":40},{"color":"Red","column":5,"row":4,"index":25},{"color":"Yellow","column":5,"row":3,"index":18},{"color":"Red","column":5,"row":2,"index":11},{"color":"Yellow","column":5,"row":1,"index":4},{"color":"Red","column":2,"row":5,"index":29},{"color":"Yellow","column":2,"row":4,"index":22},{"color":"Red","column":2,"row":3,"index":15},{"color":"Yellow","column":2,"row":2,"index":8},{"color":"Red","column":2,"row":1,"index":1},{"color":"Yellow","column":6,"row":5,"index":33},{"color":"Red","column":1,"row":6,"index":35},{"color":"Yellow","column":6,"row":4,"index":26},{"color":"Red","column":6,"row":3,"index":19},{"color":"Yellow","column":6,"row":2,"index":12},{"color":"Red","column":6,"row":1,"index":5},{"color":"Yellow","column":1,"row":5,"index":28},{"color":"Red","column":1,"row":4,"index":21},{"color":"Yellow","column":1,"row":3,"index":14},{"color":"Red","column":1,"row":2,"index":7},{"color":"Yellow","column":1,"row":1,"index":0},{"color":"Red","column":7,"row":6,"index":41},{"color":"Yellow","column":7,"row":5,"index":34},{"color":"Red","column":7,"row":4,"index":27},{"color":"Yellow","column":7,"row":3,"index":20},{"color":"Red","column":7,"row":2,"index":13},{"color":"Yellow","column":7,"row":1,"index":6}]</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-01-06T10:00:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>seed-jordan-07</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Red wins</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>["","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","Yellow","Red","Red","Red","Red","","Yellow","Yellow"]</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":1,"row":6,"index":35},{"color":"Yellow","column":7,"row":6,"index":41},{"color":"Red","column":2,"row":6,"index":36},{"color":"Yellow","column":7,"row":5,"index":34},{"color":"Red","column":3,"row":6,"index":37},{"color":"Yellow","column":6,"row":6,"index":40},{"color":"Red","column":4,"row":6,"index":38}]</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-01-07T10:00:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>seed-jordan-08</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Yellow wins</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>["","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","Red","Red","Yellow","Yellow","Yellow","Yellow","","Red","Red"]</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":7,"row":6,"index":41},{"color":"Yellow","column":1,"row":6,"index":35},{"color":"Red","column":7,"row":5,"index":34},{"color":"Yellow","column":2,"row":6,"index":36},{"color":"Red","column":6,"row":6,"index":40},{"color":"Yellow","column":3,"row":6,"index":37},{"color":"Red","column":6,"row":5,"index":33},{"color":"Yellow","column":4,"row":6,"index":38}]</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-01-08T10:00:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>seed-jordan-09</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Draw</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>["Yellow","Red","Yellow","Yellow","Yellow","Red","Yellow","Red","Yellow","Red","Red","Red","Yellow","Red","Yellow","Red","Yellow","Yellow","Yellow","Red","Yellow","Red","Yellow","Red","Red","Red","Yellow","Red","Yellow","Red","Yellow","Yellow","Red","Yellow","Yellow","Red","Yellow","Red","Red","Red","Yellow","Red"]</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":4,"row":6,"index":38},{"color":"Yellow","column":4,"row":5,"index":31},{"color":"Red","column":4,"row":4,"index":24},{"color":"Yellow","column":4,"row":3,"index":17},{"color":"Red","column":4,"row":2,"index":10},{"color":"Yellow","column":4,"row":1,"index":3},{"color":"Red","column":3,"row":6,"index":37},{"color":"Yellow","column":3,"row":5,"index":30},{"color":"Red","column":3,"row":4,"index":23},{"color":"Yellow","column":3,"row":3,"index":16},{"color":"Red","column":3,"row":2,"index":9},{"color":"Yellow","column":3,"row":1,"index":2},{"color":"Red","column":5,"row":6,"index":39},{"color":"Yellow","column":2,"row":6,"index":36},{"color":"Red","column":5,"row":5,"index":32},{"color":"Yellow","column":6,"row":6,"index":40},{"color":"Red","column":5,"row":4,"index":25},{"color":"Yellow","column":5,"row":3,"index":18},{"color":"Red","column":5,"row":2,"index":11},{"color":"Yellow","column":5,"row":1,"index":4},{"color":"Red","column":2,"row":5,"index":29},{"color":"Yellow","column":2,"row":4,"index":22},{"color":"Red","column":2,"row":3,"index":15},{"color":"Yellow","column":2,"row":2,"index":8},{"color":"Red","column":2,"row":1,"index":1},{"color":"Yellow","column":6,"row":5,"index":33},{"color":"Red","column":1,"row":6,"index":35},{"color":"Yellow","column":6,"row":4,"index":26},{"color":"Red","column":6,"row":3,"index":19},{"color":"Yellow","column":6,"row":2,"index":12},{"color":"Red","column":6,"row":1,"index":5},{"color":"Yellow","column":1,"row":5,"index":28},{"color":"Red","column":1,"row":4,"index":21},{"color":"Yellow","column":1,"row":3,"index":14},{"color":"Red","column":1,"row":2,"index":7},{"color":"Yellow","column":1,"row":1,"index":0},{"color":"Red","column":7,"row":6,"index":41},{"color":"Yellow","column":7,"row":5,"index":34},{"color":"Red","column":7,"row":4,"index":27},{"color":"Yellow","column":7,"row":3,"index":20},{"color":"Red","column":7,"row":2,"index":13},{"color":"Yellow","column":7,"row":1,"index":6}]</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-01-09T10:00:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>seed-jordan-10</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Red wins</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>["","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","Yellow","Red","Red","Red","Red","","Yellow","Yellow"]</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":1,"row":6,"index":35},{"color":"Yellow","column":7,"row":6,"index":41},{"color":"Red","column":2,"row":6,"index":36},{"color":"Yellow","column":7,"row":5,"index":34},{"color":"Red","column":3,"row":6,"index":37},{"color":"Yellow","column":6,"row":6,"index":40},{"color":"Red","column":4,"row":6,"index":38}]</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-01-10T10:00:00.000Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>jordan@dropline.test</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>seed-jordan-11</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Yellow wins</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>["","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","","Red","Red","Yellow","Yellow","Yellow","Yellow","","Red","Red"]</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>[{"color":"Red","column":7,"row":6,"index":41},{"color":"Yellow","column":1,"row":6,"index":35},{"color":"Red","column":7,"row":5,"index":34},{"color":"Yellow","column":2,"row":6,"index":36},{"color":"Red","column":6,"row":6,"index":40},{"color":"Yellow","column":3,"row":6,"index":37},{"color":"Red","column":6,"row":5,"index":33},{"color":"Yellow","column":4,"row":6,"index":38}]</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-01-11T10:00:00.000Z</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>